<commit_message>
Add table of contents to QA and update readme
</commit_message>
<xml_diff>
--- a/Documents/QA-14.xlsx
+++ b/Documents/QA-14.xlsx
@@ -8,13 +8,26 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\SCHOOL\14\sprint-10th-grade-14\Documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{168FD986-AC6C-41CD-907A-A2FD7BC65292}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{618FF72F-F534-4EDD-8FB7-0AA6B45B5F10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{A38E8662-0E47-4562-A180-E031DDA3EBF7}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="1" xr2:uid="{A38E8662-0E47-4562-A180-E031DDA3EBF7}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Table of Contents" sheetId="2" r:id="rId2"/>
   </sheets>
+  <definedNames>
+    <definedName name="_1._Application_Core_Module">Sheet1!#REF!</definedName>
+    <definedName name="_10._UI_Components_Module">Sheet1!$A$69</definedName>
+    <definedName name="_2._Main_Menu_Module">Sheet1!$A$9</definedName>
+    <definedName name="_3._Story_Module">Sheet1!$A$16</definedName>
+    <definedName name="_4._Size_Selection_Module">Sheet1!$A$24</definedName>
+    <definedName name="_5._Game_Core_Module">Sheet1!$A$34</definedName>
+    <definedName name="_6._Maze_Generation_Module">Sheet1!$A$47</definedName>
+    <definedName name="_7._Player_Module">Sheet1!$A$53</definedName>
+    <definedName name="_8._Timer_System_Module">Sheet1!$A$57</definedName>
+    <definedName name="_9._File_Persistence_Module">Sheet1!$A$65</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -36,7 +49,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="438" uniqueCount="272">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="449" uniqueCount="282">
   <si>
     <t>Test ID</t>
   </si>
@@ -107,9 +120,6 @@
     <t>Clean shutdown, return NIL state</t>
   </si>
   <si>
-    <t>APP_005</t>
-  </si>
-  <si>
     <t>Destructor</t>
   </si>
   <si>
@@ -852,13 +862,46 @@
   </si>
   <si>
     <t>QA Test Plan - 14</t>
+  </si>
+  <si>
+    <t>APP_002</t>
+  </si>
+  <si>
+    <t>Table of Contents</t>
+  </si>
+  <si>
+    <t>_2._Main_Menu_Module</t>
+  </si>
+  <si>
+    <t>_3._Story_Module</t>
+  </si>
+  <si>
+    <t>_4._Size_Selection_Module</t>
+  </si>
+  <si>
+    <t>_5._Game_Core_Module</t>
+  </si>
+  <si>
+    <t>_6._Maze_Generation_Module</t>
+  </si>
+  <si>
+    <t>_7._Player_Module</t>
+  </si>
+  <si>
+    <t>_8._Timer_System_Module</t>
+  </si>
+  <si>
+    <t>_9._File_Persistence_Module</t>
+  </si>
+  <si>
+    <t>_10._UI_Components_Module</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -897,6 +940,29 @@
       <color theme="1"/>
       <name val="Segoe UI"/>
       <family val="2"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="14"/>
+      <color theme="1"/>
+      <name val="Segoe UI"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="18"/>
+      <color theme="10"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="7">
@@ -937,7 +1003,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="27">
+  <borders count="24">
     <border>
       <left/>
       <right/>
@@ -1014,52 +1080,7 @@
     </border>
     <border>
       <left style="thin">
-        <color theme="2"/>
-      </left>
-      <right style="thin">
-        <color theme="2"/>
-      </right>
-      <top style="thin">
         <color theme="1"/>
-      </top>
-      <bottom style="thin">
-        <color theme="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color theme="1"/>
-      </left>
-      <right style="thin">
-        <color theme="1"/>
-      </right>
-      <top style="thin">
-        <color theme="1"/>
-      </top>
-      <bottom style="thin">
-        <color theme="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color theme="1"/>
-      </left>
-      <right style="thin">
-        <color theme="2"/>
-      </right>
-      <top style="thin">
-        <color theme="1"/>
-      </top>
-      <bottom style="thin">
-        <color theme="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color theme="2"/>
       </left>
       <right style="thin">
         <color theme="1"/>
@@ -1284,10 +1305,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="50">
+  <cellXfs count="47">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
@@ -1299,70 +1321,68 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="12" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="15" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="19" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="22" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="25" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
@@ -1372,48 +1392,46 @@
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="26" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="23" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="6" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="6" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -1746,10 +1764,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9CAD7174-E7B9-46BF-BD4C-618694809F80}">
-  <dimension ref="A1:K644"/>
+  <dimension ref="A1:J644"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="15.28515625" style="33" customWidth="1"/>
+    <col min="1" max="1" width="15.28515625" style="31" customWidth="1"/>
     <col min="2" max="2" width="10.28515625" customWidth="1"/>
     <col min="3" max="3" width="34.7109375" customWidth="1"/>
     <col min="4" max="4" width="26.140625" customWidth="1"/>
@@ -1760,65 +1778,65 @@
     <col min="14" max="18" width="9.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="26.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="49" t="s">
-        <v>271</v>
-      </c>
-      <c r="B1" s="49"/>
-      <c r="C1" s="49"/>
-      <c r="D1" s="49"/>
-      <c r="E1" s="49"/>
-      <c r="F1" s="49"/>
-      <c r="G1" s="49"/>
-      <c r="H1" s="17"/>
-    </row>
-    <row r="2" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="49"/>
-      <c r="B2" s="49"/>
-      <c r="C2" s="49"/>
-      <c r="D2" s="49"/>
-      <c r="E2" s="49"/>
-      <c r="F2" s="49"/>
-      <c r="G2" s="49"/>
-      <c r="H2" s="17"/>
-    </row>
-    <row r="3" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="46" t="s">
-        <v>27</v>
-      </c>
-      <c r="B3" s="47"/>
-      <c r="C3" s="47"/>
-      <c r="D3" s="47"/>
-      <c r="E3" s="47"/>
-      <c r="F3" s="47"/>
-      <c r="G3" s="48"/>
-    </row>
-    <row r="4" spans="1:11" ht="33" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10" ht="26.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="41" t="s">
+        <v>270</v>
+      </c>
+      <c r="B1" s="41"/>
+      <c r="C1" s="41"/>
+      <c r="D1" s="41"/>
+      <c r="E1" s="41"/>
+      <c r="F1" s="41"/>
+      <c r="G1" s="41"/>
+      <c r="H1" s="13"/>
+    </row>
+    <row r="2" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="41"/>
+      <c r="B2" s="41"/>
+      <c r="C2" s="41"/>
+      <c r="D2" s="41"/>
+      <c r="E2" s="41"/>
+      <c r="F2" s="41"/>
+      <c r="G2" s="41"/>
+      <c r="H2" s="13"/>
+    </row>
+    <row r="3" spans="1:10" ht="45.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="36" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" s="36" t="s">
+        <v>1</v>
+      </c>
+      <c r="C3" s="36" t="s">
+        <v>2</v>
+      </c>
+      <c r="D3" s="36" t="s">
+        <v>3</v>
+      </c>
+      <c r="E3" s="36" t="s">
+        <v>4</v>
+      </c>
+      <c r="F3" s="36" t="s">
+        <v>5</v>
+      </c>
+      <c r="G3" s="37" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="38" t="s">
-        <v>0</v>
-      </c>
-      <c r="B4" s="38" t="s">
-        <v>1</v>
-      </c>
-      <c r="C4" s="38" t="s">
-        <v>2</v>
-      </c>
-      <c r="D4" s="38" t="s">
-        <v>3</v>
-      </c>
-      <c r="E4" s="38" t="s">
-        <v>4</v>
-      </c>
-      <c r="F4" s="38" t="s">
-        <v>5</v>
-      </c>
-      <c r="G4" s="39" t="s">
-        <v>6</v>
-      </c>
+        <v>26</v>
+      </c>
+      <c r="B4" s="38"/>
+      <c r="C4" s="38"/>
+      <c r="D4" s="38"/>
+      <c r="E4" s="38"/>
+      <c r="F4" s="38"/>
+      <c r="G4" s="39"/>
       <c r="H4" s="16"/>
     </row>
-    <row r="5" spans="1:11" ht="82.5" x14ac:dyDescent="0.25">
-      <c r="A5" s="34" t="s">
+    <row r="5" spans="1:10" ht="33" x14ac:dyDescent="0.25">
+      <c r="A5" s="32" t="s">
         <v>7</v>
       </c>
       <c r="B5" s="2" t="s">
@@ -1840,11 +1858,11 @@
         <v>13</v>
       </c>
       <c r="H5" s="4"/>
-      <c r="J5" s="28"/>
-    </row>
-    <row r="6" spans="1:11" ht="66" x14ac:dyDescent="0.25">
-      <c r="A6" s="34" t="s">
-        <v>14</v>
+      <c r="J5" s="26"/>
+    </row>
+    <row r="6" spans="1:10" ht="33" x14ac:dyDescent="0.25">
+      <c r="A6" s="33" t="s">
+        <v>271</v>
       </c>
       <c r="B6" s="2" t="s">
         <v>8</v>
@@ -1866,11 +1884,11 @@
       </c>
       <c r="H6" s="4"/>
       <c r="I6" s="8"/>
-      <c r="J6" s="31"/>
-    </row>
-    <row r="7" spans="1:11" ht="66" x14ac:dyDescent="0.25">
-      <c r="A7" s="35" t="s">
-        <v>19</v>
+      <c r="J6" s="29"/>
+    </row>
+    <row r="7" spans="1:10" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="33" t="s">
+        <v>14</v>
       </c>
       <c r="B7" s="1" t="s">
         <v>8</v>
@@ -1891,1488 +1909,1487 @@
         <v>13</v>
       </c>
       <c r="H7" s="4"/>
-      <c r="J7" s="28"/>
-      <c r="K7" s="27"/>
-    </row>
-    <row r="8" spans="1:11" ht="57.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="34" t="s">
-        <v>23</v>
+      <c r="J7" s="26"/>
+    </row>
+    <row r="8" spans="1:10" ht="57.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="33" t="s">
+        <v>19</v>
       </c>
       <c r="B8" s="2" t="s">
         <v>8</v>
       </c>
       <c r="C8" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="D8" s="2" t="s">
         <v>24</v>
-      </c>
-      <c r="D8" s="2" t="s">
-        <v>25</v>
       </c>
       <c r="E8" s="2" t="s">
         <v>17</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="G8" s="20" t="s">
-        <v>13</v>
-      </c>
-      <c r="H8" s="19"/>
+        <v>25</v>
+      </c>
+      <c r="G8" s="19" t="s">
+        <v>13</v>
+      </c>
+      <c r="H8" s="18"/>
       <c r="J8" s="3"/>
     </row>
-    <row r="9" spans="1:11" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="40" t="s">
+    <row r="9" spans="1:10" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="38" t="s">
+        <v>27</v>
+      </c>
+      <c r="B9" s="38"/>
+      <c r="C9" s="38"/>
+      <c r="D9" s="38"/>
+      <c r="E9" s="38"/>
+      <c r="F9" s="38"/>
+      <c r="G9" s="39"/>
+      <c r="H9" s="13"/>
+    </row>
+    <row r="10" spans="1:10" ht="33" x14ac:dyDescent="0.25">
+      <c r="A10" s="34" t="s">
         <v>28</v>
       </c>
-      <c r="B9" s="40"/>
-      <c r="C9" s="40"/>
-      <c r="D9" s="40"/>
-      <c r="E9" s="40"/>
-      <c r="F9" s="40"/>
-      <c r="G9" s="41"/>
-      <c r="H9" s="17"/>
-    </row>
-    <row r="10" spans="1:11" ht="66" x14ac:dyDescent="0.25">
-      <c r="A10" s="36" t="s">
+      <c r="B10" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="B10" s="5" t="s">
+      <c r="C10" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="C10" s="5" t="s">
+      <c r="D10" s="5" t="s">
         <v>31</v>
-      </c>
-      <c r="D10" s="5" t="s">
-        <v>32</v>
       </c>
       <c r="E10" s="5" t="s">
         <v>17</v>
       </c>
       <c r="F10" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="G10" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="H10" s="4"/>
+    </row>
+    <row r="11" spans="1:10" ht="33" x14ac:dyDescent="0.25">
+      <c r="A11" s="30" t="s">
         <v>33</v>
       </c>
-      <c r="G10" s="11" t="s">
-        <v>13</v>
-      </c>
-      <c r="H10" s="4"/>
-    </row>
-    <row r="11" spans="1:11" ht="66" x14ac:dyDescent="0.25">
-      <c r="A11" s="32" t="s">
+      <c r="B11" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="C11" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="D11" s="6" t="s">
         <v>34</v>
       </c>
-      <c r="B11" s="6" t="s">
+      <c r="E11" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="F11" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="G11" s="14" t="s">
+        <v>13</v>
+      </c>
+      <c r="H11" s="18"/>
+    </row>
+    <row r="12" spans="1:10" ht="33" x14ac:dyDescent="0.25">
+      <c r="A12" s="30" t="s">
+        <v>37</v>
+      </c>
+      <c r="B12" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="C12" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="C11" s="6" t="s">
-        <v>31</v>
-      </c>
-      <c r="D11" s="6" t="s">
-        <v>35</v>
-      </c>
-      <c r="E11" s="6" t="s">
-        <v>36</v>
-      </c>
-      <c r="F11" s="6" t="s">
-        <v>37</v>
-      </c>
-      <c r="G11" s="14" t="s">
-        <v>13</v>
-      </c>
-      <c r="H11" s="19"/>
-    </row>
-    <row r="12" spans="1:11" ht="49.5" x14ac:dyDescent="0.25">
-      <c r="A12" s="32" t="s">
+      <c r="D12" s="6" t="s">
         <v>38</v>
       </c>
-      <c r="B12" s="6" t="s">
+      <c r="E12" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="F12" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="G12" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="H12" s="4"/>
+    </row>
+    <row r="13" spans="1:10" ht="33" x14ac:dyDescent="0.25">
+      <c r="A13" s="34" t="s">
+        <v>41</v>
+      </c>
+      <c r="B13" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="C13" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="C12" s="6" t="s">
-        <v>31</v>
-      </c>
-      <c r="D12" s="6" t="s">
-        <v>39</v>
-      </c>
-      <c r="E12" s="6" t="s">
-        <v>40</v>
-      </c>
-      <c r="F12" s="6" t="s">
-        <v>41</v>
-      </c>
-      <c r="G12" s="12" t="s">
-        <v>13</v>
-      </c>
-      <c r="H12" s="4"/>
-    </row>
-    <row r="13" spans="1:11" ht="66" x14ac:dyDescent="0.25">
-      <c r="A13" s="36" t="s">
+      <c r="D13" s="5" t="s">
         <v>42</v>
       </c>
-      <c r="B13" s="5" t="s">
+      <c r="E13" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="F13" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="G13" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="H13" s="4"/>
+    </row>
+    <row r="14" spans="1:10" ht="66" x14ac:dyDescent="0.25">
+      <c r="A14" s="30" t="s">
+        <v>45</v>
+      </c>
+      <c r="B14" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="C14" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="C13" s="5" t="s">
-        <v>31</v>
-      </c>
-      <c r="D13" s="5" t="s">
-        <v>43</v>
-      </c>
-      <c r="E13" s="5" t="s">
-        <v>44</v>
-      </c>
-      <c r="F13" s="5" t="s">
-        <v>45</v>
-      </c>
-      <c r="G13" s="11" t="s">
-        <v>13</v>
-      </c>
-      <c r="H13" s="4"/>
-    </row>
-    <row r="14" spans="1:11" ht="66" x14ac:dyDescent="0.25">
-      <c r="A14" s="32" t="s">
+      <c r="D14" s="6" t="s">
         <v>46</v>
-      </c>
-      <c r="B14" s="6" t="s">
-        <v>30</v>
-      </c>
-      <c r="C14" s="6" t="s">
-        <v>31</v>
-      </c>
-      <c r="D14" s="6" t="s">
-        <v>47</v>
       </c>
       <c r="E14" s="6" t="s">
         <v>17</v>
       </c>
       <c r="F14" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="G14" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="H14" s="4"/>
+    </row>
+    <row r="15" spans="1:10" ht="49.5" x14ac:dyDescent="0.25">
+      <c r="A15" s="34" t="s">
         <v>48</v>
       </c>
-      <c r="G14" s="12" t="s">
-        <v>13</v>
-      </c>
-      <c r="H14" s="4"/>
-    </row>
-    <row r="15" spans="1:11" ht="49.5" x14ac:dyDescent="0.25">
-      <c r="A15" s="36" t="s">
+      <c r="B15" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="C15" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="D15" s="5" t="s">
         <v>49</v>
-      </c>
-      <c r="B15" s="5" t="s">
-        <v>30</v>
-      </c>
-      <c r="C15" s="5" t="s">
-        <v>31</v>
-      </c>
-      <c r="D15" s="5" t="s">
-        <v>50</v>
       </c>
       <c r="E15" s="5" t="s">
         <v>17</v>
       </c>
       <c r="F15" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="G15" s="20" t="s">
+        <v>13</v>
+      </c>
+      <c r="H15" s="13"/>
+    </row>
+    <row r="16" spans="1:10" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="40" t="s">
         <v>51</v>
       </c>
-      <c r="G15" s="21" t="s">
-        <v>13</v>
-      </c>
-      <c r="H15" s="17"/>
-    </row>
-    <row r="16" spans="1:11" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="42" t="s">
+      <c r="B16" s="40"/>
+      <c r="C16" s="40"/>
+      <c r="D16" s="40"/>
+      <c r="E16" s="40"/>
+      <c r="F16" s="40"/>
+      <c r="G16" s="40"/>
+      <c r="H16" s="27"/>
+    </row>
+    <row r="17" spans="1:8" ht="66" x14ac:dyDescent="0.25">
+      <c r="A17" s="34" t="s">
         <v>52</v>
       </c>
-      <c r="B16" s="42"/>
-      <c r="C16" s="42"/>
-      <c r="D16" s="42"/>
-      <c r="E16" s="42"/>
-      <c r="F16" s="42"/>
-      <c r="G16" s="42"/>
-      <c r="H16" s="29"/>
-    </row>
-    <row r="17" spans="1:8" ht="66" x14ac:dyDescent="0.25">
-      <c r="A17" s="36" t="s">
+      <c r="B17" s="5" t="s">
         <v>53</v>
       </c>
-      <c r="B17" s="5" t="s">
+      <c r="C17" s="5" t="s">
         <v>54</v>
       </c>
-      <c r="C17" s="5" t="s">
+      <c r="D17" s="5" t="s">
         <v>55</v>
-      </c>
-      <c r="D17" s="5" t="s">
-        <v>56</v>
       </c>
       <c r="E17" s="5" t="s">
         <v>17</v>
       </c>
       <c r="F17" s="5" t="s">
+        <v>56</v>
+      </c>
+      <c r="G17" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="H17" s="4"/>
+    </row>
+    <row r="18" spans="1:8" ht="49.5" x14ac:dyDescent="0.25">
+      <c r="A18" s="30" t="s">
         <v>57</v>
       </c>
-      <c r="G17" s="11" t="s">
-        <v>13</v>
-      </c>
-      <c r="H17" s="4"/>
-    </row>
-    <row r="18" spans="1:8" ht="49.5" x14ac:dyDescent="0.25">
-      <c r="A18" s="32" t="s">
+      <c r="B18" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="C18" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="D18" s="6" t="s">
         <v>58</v>
       </c>
-      <c r="B18" s="6" t="s">
+      <c r="E18" s="6" t="s">
+        <v>59</v>
+      </c>
+      <c r="F18" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="G18" s="21" t="s">
+        <v>13</v>
+      </c>
+      <c r="H18" s="18"/>
+    </row>
+    <row r="19" spans="1:8" ht="66" x14ac:dyDescent="0.25">
+      <c r="A19" s="30" t="s">
+        <v>61</v>
+      </c>
+      <c r="B19" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="C19" s="6" t="s">
         <v>54</v>
       </c>
-      <c r="C18" s="6" t="s">
-        <v>55</v>
-      </c>
-      <c r="D18" s="6" t="s">
-        <v>59</v>
-      </c>
-      <c r="E18" s="6" t="s">
-        <v>60</v>
-      </c>
-      <c r="F18" s="6" t="s">
-        <v>61</v>
-      </c>
-      <c r="G18" s="22" t="s">
-        <v>13</v>
-      </c>
-      <c r="H18" s="19"/>
-    </row>
-    <row r="19" spans="1:8" ht="66" x14ac:dyDescent="0.25">
-      <c r="A19" s="32" t="s">
+      <c r="D19" s="6" t="s">
         <v>62</v>
       </c>
-      <c r="B19" s="6" t="s">
+      <c r="E19" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="F19" s="6" t="s">
+        <v>64</v>
+      </c>
+      <c r="G19" s="22" t="s">
+        <v>13</v>
+      </c>
+      <c r="H19" s="4"/>
+    </row>
+    <row r="20" spans="1:8" ht="49.5" x14ac:dyDescent="0.25">
+      <c r="A20" s="34" t="s">
+        <v>65</v>
+      </c>
+      <c r="B20" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="C20" s="5" t="s">
         <v>54</v>
       </c>
-      <c r="C19" s="6" t="s">
-        <v>55</v>
-      </c>
-      <c r="D19" s="6" t="s">
-        <v>63</v>
-      </c>
-      <c r="E19" s="6" t="s">
-        <v>64</v>
-      </c>
-      <c r="F19" s="6" t="s">
-        <v>65</v>
-      </c>
-      <c r="G19" s="23" t="s">
-        <v>13</v>
-      </c>
-      <c r="H19" s="4"/>
-    </row>
-    <row r="20" spans="1:8" ht="49.5" x14ac:dyDescent="0.25">
-      <c r="A20" s="36" t="s">
+      <c r="D20" s="5" t="s">
         <v>66</v>
       </c>
-      <c r="B20" s="5" t="s">
-        <v>54</v>
-      </c>
-      <c r="C20" s="5" t="s">
-        <v>55</v>
-      </c>
-      <c r="D20" s="5" t="s">
+      <c r="E20" s="5" t="s">
         <v>67</v>
       </c>
-      <c r="E20" s="5" t="s">
+      <c r="F20" s="5" t="s">
         <v>68</v>
       </c>
-      <c r="F20" s="5" t="s">
+      <c r="G20" s="20" t="s">
+        <v>13</v>
+      </c>
+      <c r="H20" s="18"/>
+    </row>
+    <row r="21" spans="1:8" ht="82.5" x14ac:dyDescent="0.25">
+      <c r="A21" s="30" t="s">
         <v>69</v>
       </c>
-      <c r="G20" s="21" t="s">
-        <v>13</v>
-      </c>
-      <c r="H20" s="19"/>
-    </row>
-    <row r="21" spans="1:8" ht="82.5" x14ac:dyDescent="0.25">
-      <c r="A21" s="32" t="s">
+      <c r="B21" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="C21" s="6" t="s">
         <v>70</v>
       </c>
-      <c r="B21" s="6" t="s">
-        <v>54</v>
-      </c>
-      <c r="C21" s="6" t="s">
+      <c r="D21" s="6" t="s">
         <v>71</v>
-      </c>
-      <c r="D21" s="6" t="s">
-        <v>72</v>
       </c>
       <c r="E21" s="6" t="s">
         <v>17</v>
       </c>
       <c r="F21" s="6" t="s">
+        <v>72</v>
+      </c>
+      <c r="G21" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="H21" s="4"/>
+    </row>
+    <row r="22" spans="1:8" ht="82.5" x14ac:dyDescent="0.25">
+      <c r="A22" s="34" t="s">
         <v>73</v>
       </c>
-      <c r="G21" s="12" t="s">
-        <v>13</v>
-      </c>
-      <c r="H21" s="4"/>
-    </row>
-    <row r="22" spans="1:8" ht="82.5" x14ac:dyDescent="0.25">
-      <c r="A22" s="36" t="s">
+      <c r="B22" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="C22" s="5" t="s">
+        <v>70</v>
+      </c>
+      <c r="D22" s="5" t="s">
         <v>74</v>
-      </c>
-      <c r="B22" s="5" t="s">
-        <v>54</v>
-      </c>
-      <c r="C22" s="5" t="s">
-        <v>71</v>
-      </c>
-      <c r="D22" s="5" t="s">
-        <v>75</v>
       </c>
       <c r="E22" s="5" t="s">
         <v>17</v>
       </c>
       <c r="F22" s="5" t="s">
+        <v>75</v>
+      </c>
+      <c r="G22" s="20" t="s">
+        <v>13</v>
+      </c>
+      <c r="H22" s="18"/>
+    </row>
+    <row r="23" spans="1:8" ht="33" x14ac:dyDescent="0.25">
+      <c r="A23" s="34" t="s">
         <v>76</v>
       </c>
-      <c r="G22" s="21" t="s">
-        <v>13</v>
-      </c>
-      <c r="H22" s="19"/>
-    </row>
-    <row r="23" spans="1:8" ht="33" x14ac:dyDescent="0.25">
-      <c r="A23" s="36" t="s">
+      <c r="B23" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="C23" s="5" t="s">
+        <v>70</v>
+      </c>
+      <c r="D23" s="5" t="s">
         <v>77</v>
-      </c>
-      <c r="B23" s="5" t="s">
-        <v>54</v>
-      </c>
-      <c r="C23" s="5" t="s">
-        <v>71</v>
-      </c>
-      <c r="D23" s="5" t="s">
-        <v>78</v>
       </c>
       <c r="E23" s="5" t="s">
         <v>17</v>
       </c>
       <c r="F23" s="5" t="s">
+        <v>78</v>
+      </c>
+      <c r="G23" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="H23" s="4"/>
+    </row>
+    <row r="24" spans="1:8" ht="32.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="40" t="s">
         <v>79</v>
       </c>
-      <c r="G23" s="11" t="s">
-        <v>13</v>
-      </c>
-      <c r="H23" s="4"/>
-    </row>
-    <row r="24" spans="1:8" ht="32.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="42" t="s">
+      <c r="B24" s="40"/>
+      <c r="C24" s="40"/>
+      <c r="D24" s="40"/>
+      <c r="E24" s="40"/>
+      <c r="F24" s="40"/>
+      <c r="G24" s="40"/>
+      <c r="H24" s="27"/>
+    </row>
+    <row r="25" spans="1:8" ht="66" x14ac:dyDescent="0.25">
+      <c r="A25" s="34" t="s">
         <v>80</v>
       </c>
-      <c r="B24" s="42"/>
-      <c r="C24" s="42"/>
-      <c r="D24" s="42"/>
-      <c r="E24" s="42"/>
-      <c r="F24" s="42"/>
-      <c r="G24" s="42"/>
-      <c r="H24" s="29"/>
-    </row>
-    <row r="25" spans="1:8" ht="66" x14ac:dyDescent="0.25">
-      <c r="A25" s="36" t="s">
+      <c r="B25" s="5" t="s">
         <v>81</v>
       </c>
-      <c r="B25" s="5" t="s">
+      <c r="C25" s="5" t="s">
         <v>82</v>
       </c>
-      <c r="C25" s="5" t="s">
+      <c r="D25" s="5" t="s">
         <v>83</v>
-      </c>
-      <c r="D25" s="5" t="s">
-        <v>84</v>
       </c>
       <c r="E25" s="5" t="s">
         <v>17</v>
       </c>
       <c r="F25" s="5" t="s">
+        <v>84</v>
+      </c>
+      <c r="G25" s="20" t="s">
+        <v>13</v>
+      </c>
+      <c r="H25" s="23"/>
+    </row>
+    <row r="26" spans="1:8" ht="66" x14ac:dyDescent="0.25">
+      <c r="A26" s="30" t="s">
         <v>85</v>
       </c>
-      <c r="G25" s="21" t="s">
-        <v>13</v>
-      </c>
-      <c r="H25" s="24"/>
-    </row>
-    <row r="26" spans="1:8" ht="66" x14ac:dyDescent="0.25">
-      <c r="A26" s="32" t="s">
+      <c r="B26" s="6" t="s">
+        <v>81</v>
+      </c>
+      <c r="C26" s="6" t="s">
+        <v>82</v>
+      </c>
+      <c r="D26" s="6" t="s">
         <v>86</v>
       </c>
-      <c r="B26" s="6" t="s">
+      <c r="E26" s="6" t="s">
+        <v>87</v>
+      </c>
+      <c r="F26" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="G26" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="H26" s="15"/>
+    </row>
+    <row r="27" spans="1:8" ht="82.5" x14ac:dyDescent="0.25">
+      <c r="A27" s="30" t="s">
+        <v>89</v>
+      </c>
+      <c r="B27" s="6" t="s">
+        <v>81</v>
+      </c>
+      <c r="C27" s="6" t="s">
         <v>82</v>
       </c>
-      <c r="C26" s="6" t="s">
-        <v>83</v>
-      </c>
-      <c r="D26" s="6" t="s">
-        <v>87</v>
-      </c>
-      <c r="E26" s="6" t="s">
-        <v>88</v>
-      </c>
-      <c r="F26" s="6" t="s">
-        <v>89</v>
-      </c>
-      <c r="G26" s="12" t="s">
-        <v>13</v>
-      </c>
-      <c r="H26" s="15"/>
-    </row>
-    <row r="27" spans="1:8" ht="82.5" x14ac:dyDescent="0.25">
-      <c r="A27" s="32" t="s">
+      <c r="D27" s="6" t="s">
         <v>90</v>
       </c>
-      <c r="B27" s="6" t="s">
+      <c r="E27" s="6" t="s">
+        <v>91</v>
+      </c>
+      <c r="F27" s="6" t="s">
+        <v>92</v>
+      </c>
+      <c r="G27" s="14" t="s">
+        <v>13</v>
+      </c>
+      <c r="H27" s="17"/>
+    </row>
+    <row r="28" spans="1:8" ht="66" x14ac:dyDescent="0.25">
+      <c r="A28" s="34" t="s">
+        <v>93</v>
+      </c>
+      <c r="B28" s="5" t="s">
+        <v>81</v>
+      </c>
+      <c r="C28" s="5" t="s">
         <v>82</v>
       </c>
-      <c r="C27" s="6" t="s">
-        <v>83</v>
-      </c>
-      <c r="D27" s="6" t="s">
-        <v>91</v>
-      </c>
-      <c r="E27" s="6" t="s">
-        <v>92</v>
-      </c>
-      <c r="F27" s="6" t="s">
-        <v>93</v>
-      </c>
-      <c r="G27" s="14" t="s">
-        <v>13</v>
-      </c>
-      <c r="H27" s="18"/>
-    </row>
-    <row r="28" spans="1:8" ht="66" x14ac:dyDescent="0.25">
-      <c r="A28" s="36" t="s">
+      <c r="D28" s="5" t="s">
         <v>94</v>
       </c>
-      <c r="B28" s="5" t="s">
+      <c r="E28" s="5" t="s">
+        <v>95</v>
+      </c>
+      <c r="F28" s="5" t="s">
+        <v>96</v>
+      </c>
+      <c r="G28" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="H28" s="24"/>
+    </row>
+    <row r="29" spans="1:8" ht="33" x14ac:dyDescent="0.25">
+      <c r="A29" s="30" t="s">
+        <v>97</v>
+      </c>
+      <c r="B29" s="6" t="s">
+        <v>81</v>
+      </c>
+      <c r="C29" s="6" t="s">
         <v>82</v>
       </c>
-      <c r="C28" s="5" t="s">
-        <v>83</v>
-      </c>
-      <c r="D28" s="5" t="s">
-        <v>95</v>
-      </c>
-      <c r="E28" s="5" t="s">
-        <v>96</v>
-      </c>
-      <c r="F28" s="5" t="s">
-        <v>97</v>
-      </c>
-      <c r="G28" s="11" t="s">
-        <v>13</v>
-      </c>
-      <c r="H28" s="25"/>
-    </row>
-    <row r="29" spans="1:8" ht="33" x14ac:dyDescent="0.25">
-      <c r="A29" s="32" t="s">
+      <c r="D29" s="6" t="s">
         <v>98</v>
       </c>
-      <c r="B29" s="6" t="s">
+      <c r="E29" s="6" t="s">
+        <v>99</v>
+      </c>
+      <c r="F29" s="6" t="s">
+        <v>100</v>
+      </c>
+      <c r="G29" s="14" t="s">
+        <v>13</v>
+      </c>
+      <c r="H29" s="17"/>
+    </row>
+    <row r="30" spans="1:8" ht="33" x14ac:dyDescent="0.25">
+      <c r="A30" s="34" t="s">
+        <v>101</v>
+      </c>
+      <c r="B30" s="5" t="s">
+        <v>81</v>
+      </c>
+      <c r="C30" s="5" t="s">
         <v>82</v>
       </c>
-      <c r="C29" s="6" t="s">
-        <v>83</v>
-      </c>
-      <c r="D29" s="6" t="s">
-        <v>99</v>
-      </c>
-      <c r="E29" s="6" t="s">
-        <v>100</v>
-      </c>
-      <c r="F29" s="6" t="s">
-        <v>101</v>
-      </c>
-      <c r="G29" s="14" t="s">
-        <v>13</v>
-      </c>
-      <c r="H29" s="18"/>
-    </row>
-    <row r="30" spans="1:8" ht="49.5" x14ac:dyDescent="0.25">
-      <c r="A30" s="36" t="s">
+      <c r="D30" s="5" t="s">
         <v>102</v>
-      </c>
-      <c r="B30" s="5" t="s">
-        <v>82</v>
-      </c>
-      <c r="C30" s="5" t="s">
-        <v>83</v>
-      </c>
-      <c r="D30" s="5" t="s">
-        <v>103</v>
       </c>
       <c r="E30" s="5" t="s">
         <v>17</v>
       </c>
       <c r="F30" s="5" t="s">
+        <v>103</v>
+      </c>
+      <c r="G30" s="20" t="s">
+        <v>13</v>
+      </c>
+      <c r="H30" s="23"/>
+    </row>
+    <row r="31" spans="1:8" ht="33" x14ac:dyDescent="0.25">
+      <c r="A31" s="34" t="s">
         <v>104</v>
       </c>
-      <c r="G30" s="21" t="s">
-        <v>13</v>
-      </c>
-      <c r="H30" s="24"/>
-    </row>
-    <row r="31" spans="1:8" ht="33" x14ac:dyDescent="0.25">
-      <c r="A31" s="36" t="s">
+      <c r="B31" s="5" t="s">
+        <v>81</v>
+      </c>
+      <c r="C31" s="5" t="s">
         <v>105</v>
       </c>
-      <c r="B31" s="5" t="s">
-        <v>82</v>
-      </c>
-      <c r="C31" s="5" t="s">
+      <c r="D31" s="5" t="s">
         <v>106</v>
       </c>
-      <c r="D31" s="5" t="s">
+      <c r="E31" s="5" t="s">
         <v>107</v>
       </c>
-      <c r="E31" s="5" t="s">
+      <c r="F31" s="5" t="s">
         <v>108</v>
       </c>
-      <c r="F31" s="5" t="s">
+      <c r="G31" s="20" t="s">
+        <v>13</v>
+      </c>
+      <c r="H31" s="23"/>
+    </row>
+    <row r="32" spans="1:8" ht="33" x14ac:dyDescent="0.25">
+      <c r="A32" s="34" t="s">
         <v>109</v>
       </c>
-      <c r="G31" s="21" t="s">
-        <v>13</v>
-      </c>
-      <c r="H31" s="24"/>
-    </row>
-    <row r="32" spans="1:8" ht="33" x14ac:dyDescent="0.25">
-      <c r="A32" s="36" t="s">
+      <c r="B32" s="5" t="s">
+        <v>81</v>
+      </c>
+      <c r="C32" s="5" t="s">
+        <v>105</v>
+      </c>
+      <c r="D32" s="5" t="s">
         <v>110</v>
       </c>
-      <c r="B32" s="5" t="s">
-        <v>82</v>
-      </c>
-      <c r="C32" s="5" t="s">
-        <v>106</v>
-      </c>
-      <c r="D32" s="5" t="s">
+      <c r="E32" s="5" t="s">
         <v>111</v>
       </c>
-      <c r="E32" s="5" t="s">
+      <c r="F32" s="5" t="s">
         <v>112</v>
       </c>
-      <c r="F32" s="5" t="s">
+      <c r="G32" s="20" t="s">
+        <v>13</v>
+      </c>
+      <c r="H32" s="23"/>
+    </row>
+    <row r="33" spans="1:8" ht="33" x14ac:dyDescent="0.25">
+      <c r="A33" s="30" t="s">
         <v>113</v>
       </c>
-      <c r="G32" s="21" t="s">
-        <v>13</v>
-      </c>
-      <c r="H32" s="24"/>
-    </row>
-    <row r="33" spans="1:8" ht="33" x14ac:dyDescent="0.25">
-      <c r="A33" s="32" t="s">
+      <c r="B33" s="6" t="s">
+        <v>81</v>
+      </c>
+      <c r="C33" s="6" t="s">
+        <v>105</v>
+      </c>
+      <c r="D33" s="6" t="s">
         <v>114</v>
       </c>
-      <c r="B33" s="6" t="s">
-        <v>82</v>
-      </c>
-      <c r="C33" s="6" t="s">
-        <v>106</v>
-      </c>
-      <c r="D33" s="6" t="s">
+      <c r="E33" s="6" t="s">
         <v>115</v>
       </c>
-      <c r="E33" s="6" t="s">
+      <c r="F33" s="6" t="s">
         <v>116</v>
       </c>
-      <c r="F33" s="6" t="s">
+      <c r="G33" s="28" t="s">
+        <v>13</v>
+      </c>
+      <c r="H33" s="17"/>
+    </row>
+    <row r="34" spans="1:8" ht="26.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A34" s="40" t="s">
         <v>117</v>
       </c>
-      <c r="G33" s="30" t="s">
-        <v>13</v>
-      </c>
-      <c r="H33" s="18"/>
-    </row>
-    <row r="34" spans="1:8" ht="26.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="42" t="s">
+      <c r="B34" s="40"/>
+      <c r="C34" s="40"/>
+      <c r="D34" s="40"/>
+      <c r="E34" s="40"/>
+      <c r="F34" s="40"/>
+      <c r="G34" s="40"/>
+      <c r="H34" s="27"/>
+    </row>
+    <row r="35" spans="1:8" ht="82.5" x14ac:dyDescent="0.25">
+      <c r="A35" s="30" t="s">
         <v>118</v>
       </c>
-      <c r="B34" s="42"/>
-      <c r="C34" s="42"/>
-      <c r="D34" s="42"/>
-      <c r="E34" s="42"/>
-      <c r="F34" s="42"/>
-      <c r="G34" s="42"/>
-      <c r="H34" s="29"/>
-    </row>
-    <row r="35" spans="1:8" ht="82.5" x14ac:dyDescent="0.25">
-      <c r="A35" s="32" t="s">
+      <c r="B35" s="6" t="s">
         <v>119</v>
       </c>
-      <c r="B35" s="6" t="s">
+      <c r="C35" s="6" t="s">
         <v>120</v>
       </c>
-      <c r="C35" s="6" t="s">
+      <c r="D35" s="6" t="s">
         <v>121</v>
-      </c>
-      <c r="D35" s="6" t="s">
-        <v>122</v>
       </c>
       <c r="E35" s="6" t="s">
         <v>17</v>
       </c>
       <c r="F35" s="6" t="s">
+        <v>122</v>
+      </c>
+      <c r="G35" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="H35" s="15"/>
+    </row>
+    <row r="36" spans="1:8" ht="49.5" x14ac:dyDescent="0.25">
+      <c r="A36" s="30" t="s">
         <v>123</v>
       </c>
-      <c r="G35" s="12" t="s">
-        <v>13</v>
-      </c>
-      <c r="H35" s="15"/>
-    </row>
-    <row r="36" spans="1:8" ht="49.5" x14ac:dyDescent="0.25">
-      <c r="A36" s="32" t="s">
+      <c r="B36" s="6" t="s">
+        <v>119</v>
+      </c>
+      <c r="C36" s="6" t="s">
         <v>124</v>
       </c>
-      <c r="B36" s="6" t="s">
-        <v>120</v>
-      </c>
-      <c r="C36" s="6" t="s">
+      <c r="D36" s="6" t="s">
         <v>125</v>
       </c>
-      <c r="D36" s="6" t="s">
+      <c r="E36" s="6" t="s">
+        <v>59</v>
+      </c>
+      <c r="F36" s="6" t="s">
         <v>126</v>
       </c>
-      <c r="E36" s="6" t="s">
-        <v>60</v>
-      </c>
-      <c r="F36" s="6" t="s">
+      <c r="G36" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="H36" s="15"/>
+    </row>
+    <row r="37" spans="1:8" ht="49.5" x14ac:dyDescent="0.25">
+      <c r="A37" s="30" t="s">
         <v>127</v>
       </c>
-      <c r="G36" s="12" t="s">
-        <v>13</v>
-      </c>
-      <c r="H36" s="15"/>
-    </row>
-    <row r="37" spans="1:8" ht="49.5" x14ac:dyDescent="0.25">
-      <c r="A37" s="32" t="s">
+      <c r="B37" s="6" t="s">
+        <v>119</v>
+      </c>
+      <c r="C37" s="6" t="s">
+        <v>124</v>
+      </c>
+      <c r="D37" s="6" t="s">
         <v>128</v>
       </c>
-      <c r="B37" s="6" t="s">
-        <v>120</v>
-      </c>
-      <c r="C37" s="6" t="s">
-        <v>125</v>
-      </c>
-      <c r="D37" s="6" t="s">
+      <c r="E37" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="F37" s="6" t="s">
         <v>129</v>
       </c>
-      <c r="E37" s="6" t="s">
-        <v>64</v>
-      </c>
-      <c r="F37" s="6" t="s">
+      <c r="G37" s="14" t="s">
+        <v>13</v>
+      </c>
+      <c r="H37" s="17"/>
+    </row>
+    <row r="38" spans="1:8" ht="49.5" x14ac:dyDescent="0.25">
+      <c r="A38" s="30" t="s">
         <v>130</v>
       </c>
-      <c r="G37" s="14" t="s">
-        <v>13</v>
-      </c>
-      <c r="H37" s="18"/>
-    </row>
-    <row r="38" spans="1:8" ht="49.5" x14ac:dyDescent="0.25">
-      <c r="A38" s="32" t="s">
+      <c r="B38" s="6" t="s">
+        <v>119</v>
+      </c>
+      <c r="C38" s="6" t="s">
+        <v>124</v>
+      </c>
+      <c r="D38" s="6" t="s">
         <v>131</v>
       </c>
-      <c r="B38" s="6" t="s">
-        <v>120</v>
-      </c>
-      <c r="C38" s="6" t="s">
-        <v>125</v>
-      </c>
-      <c r="D38" s="6" t="s">
+      <c r="E38" s="6" t="s">
         <v>132</v>
       </c>
-      <c r="E38" s="6" t="s">
+      <c r="F38" s="6" t="s">
         <v>133</v>
       </c>
-      <c r="F38" s="6" t="s">
+      <c r="G38" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="H38" s="15"/>
+    </row>
+    <row r="39" spans="1:8" ht="66" x14ac:dyDescent="0.25">
+      <c r="A39" s="30" t="s">
         <v>134</v>
       </c>
-      <c r="G38" s="12" t="s">
-        <v>13</v>
-      </c>
-      <c r="H38" s="15"/>
-    </row>
-    <row r="39" spans="1:8" ht="66" x14ac:dyDescent="0.25">
-      <c r="A39" s="32" t="s">
+      <c r="B39" s="6" t="s">
+        <v>119</v>
+      </c>
+      <c r="C39" s="6" t="s">
+        <v>124</v>
+      </c>
+      <c r="D39" s="6" t="s">
         <v>135</v>
       </c>
-      <c r="B39" s="6" t="s">
-        <v>120</v>
-      </c>
-      <c r="C39" s="6" t="s">
-        <v>125</v>
-      </c>
-      <c r="D39" s="6" t="s">
+      <c r="E39" s="6" t="s">
         <v>136</v>
       </c>
-      <c r="E39" s="6" t="s">
+      <c r="F39" s="6" t="s">
         <v>137</v>
       </c>
-      <c r="F39" s="6" t="s">
+      <c r="G39" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="H39" s="15"/>
+    </row>
+    <row r="40" spans="1:8" ht="49.5" x14ac:dyDescent="0.25">
+      <c r="A40" s="30" t="s">
         <v>138</v>
       </c>
-      <c r="G39" s="12" t="s">
-        <v>13</v>
-      </c>
-      <c r="H39" s="15"/>
-    </row>
-    <row r="40" spans="1:8" ht="49.5" x14ac:dyDescent="0.25">
-      <c r="A40" s="32" t="s">
+      <c r="B40" s="6" t="s">
+        <v>119</v>
+      </c>
+      <c r="C40" s="6" t="s">
+        <v>124</v>
+      </c>
+      <c r="D40" s="6" t="s">
         <v>139</v>
       </c>
-      <c r="B40" s="6" t="s">
-        <v>120</v>
-      </c>
-      <c r="C40" s="6" t="s">
-        <v>125</v>
-      </c>
-      <c r="D40" s="6" t="s">
+      <c r="E40" s="6" t="s">
         <v>140</v>
       </c>
-      <c r="E40" s="6" t="s">
+      <c r="F40" s="6" t="s">
         <v>141</v>
       </c>
-      <c r="F40" s="6" t="s">
+      <c r="G40" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="H40" s="15"/>
+    </row>
+    <row r="41" spans="1:8" ht="66" x14ac:dyDescent="0.25">
+      <c r="A41" s="30" t="s">
         <v>142</v>
       </c>
-      <c r="G40" s="12" t="s">
-        <v>13</v>
-      </c>
-      <c r="H40" s="15"/>
-    </row>
-    <row r="41" spans="1:8" ht="66" x14ac:dyDescent="0.25">
-      <c r="A41" s="32" t="s">
+      <c r="B41" s="6" t="s">
+        <v>119</v>
+      </c>
+      <c r="C41" s="6" t="s">
+        <v>124</v>
+      </c>
+      <c r="D41" s="6" t="s">
         <v>143</v>
       </c>
-      <c r="B41" s="6" t="s">
-        <v>120</v>
-      </c>
-      <c r="C41" s="6" t="s">
-        <v>125</v>
-      </c>
-      <c r="D41" s="6" t="s">
+      <c r="E41" s="6" t="s">
         <v>144</v>
       </c>
-      <c r="E41" s="6" t="s">
+      <c r="F41" s="6" t="s">
         <v>145</v>
       </c>
-      <c r="F41" s="6" t="s">
+      <c r="G41" s="14" t="s">
+        <v>13</v>
+      </c>
+      <c r="H41" s="17"/>
+    </row>
+    <row r="42" spans="1:8" ht="33" x14ac:dyDescent="0.25">
+      <c r="A42" s="30" t="s">
         <v>146</v>
       </c>
-      <c r="G41" s="14" t="s">
-        <v>13</v>
-      </c>
-      <c r="H41" s="18"/>
-    </row>
-    <row r="42" spans="1:8" ht="33" x14ac:dyDescent="0.25">
-      <c r="A42" s="32" t="s">
+      <c r="B42" s="6" t="s">
+        <v>119</v>
+      </c>
+      <c r="C42" s="6" t="s">
+        <v>124</v>
+      </c>
+      <c r="D42" s="6" t="s">
         <v>147</v>
       </c>
-      <c r="B42" s="6" t="s">
-        <v>120</v>
-      </c>
-      <c r="C42" s="6" t="s">
-        <v>125</v>
-      </c>
-      <c r="D42" s="6" t="s">
+      <c r="E42" s="6" t="s">
         <v>148</v>
       </c>
-      <c r="E42" s="6" t="s">
+      <c r="F42" s="6" t="s">
         <v>149</v>
       </c>
-      <c r="F42" s="6" t="s">
+      <c r="G42" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="H42" s="15"/>
+    </row>
+    <row r="43" spans="1:8" ht="82.5" x14ac:dyDescent="0.25">
+      <c r="A43" s="30" t="s">
         <v>150</v>
       </c>
-      <c r="G42" s="12" t="s">
-        <v>13</v>
-      </c>
-      <c r="H42" s="15"/>
-    </row>
-    <row r="43" spans="1:8" ht="82.5" x14ac:dyDescent="0.25">
-      <c r="A43" s="32" t="s">
+      <c r="B43" s="6" t="s">
+        <v>119</v>
+      </c>
+      <c r="C43" s="6" t="s">
         <v>151</v>
       </c>
-      <c r="B43" s="6" t="s">
-        <v>120</v>
-      </c>
-      <c r="C43" s="6" t="s">
+      <c r="D43" s="6" t="s">
         <v>152</v>
-      </c>
-      <c r="D43" s="6" t="s">
-        <v>153</v>
       </c>
       <c r="E43" s="6" t="s">
         <v>17</v>
       </c>
       <c r="F43" s="6" t="s">
+        <v>153</v>
+      </c>
+      <c r="G43" s="14" t="s">
+        <v>13</v>
+      </c>
+      <c r="H43" s="17"/>
+    </row>
+    <row r="44" spans="1:8" ht="66" x14ac:dyDescent="0.25">
+      <c r="A44" s="30" t="s">
         <v>154</v>
       </c>
-      <c r="G43" s="14" t="s">
-        <v>13</v>
-      </c>
-      <c r="H43" s="18"/>
-    </row>
-    <row r="44" spans="1:8" ht="66" x14ac:dyDescent="0.25">
-      <c r="A44" s="32" t="s">
+      <c r="B44" s="6" t="s">
+        <v>119</v>
+      </c>
+      <c r="C44" s="6" t="s">
+        <v>151</v>
+      </c>
+      <c r="D44" s="6" t="s">
         <v>155</v>
       </c>
-      <c r="B44" s="6" t="s">
-        <v>120</v>
-      </c>
-      <c r="C44" s="6" t="s">
-        <v>152</v>
-      </c>
-      <c r="D44" s="6" t="s">
+      <c r="E44" s="6" t="s">
         <v>156</v>
       </c>
-      <c r="E44" s="6" t="s">
+      <c r="F44" s="6" t="s">
         <v>157</v>
       </c>
-      <c r="F44" s="6" t="s">
+      <c r="G44" s="14" t="s">
+        <v>13</v>
+      </c>
+      <c r="H44" s="17"/>
+    </row>
+    <row r="45" spans="1:8" ht="49.5" x14ac:dyDescent="0.25">
+      <c r="A45" s="30" t="s">
         <v>158</v>
       </c>
-      <c r="G44" s="14" t="s">
-        <v>13</v>
-      </c>
-      <c r="H44" s="18"/>
-    </row>
-    <row r="45" spans="1:8" ht="49.5" x14ac:dyDescent="0.25">
-      <c r="A45" s="32" t="s">
+      <c r="B45" s="6" t="s">
+        <v>119</v>
+      </c>
+      <c r="C45" s="6" t="s">
         <v>159</v>
       </c>
-      <c r="B45" s="6" t="s">
-        <v>120</v>
-      </c>
-      <c r="C45" s="6" t="s">
+      <c r="D45" s="6" t="s">
         <v>160</v>
-      </c>
-      <c r="D45" s="6" t="s">
-        <v>161</v>
       </c>
       <c r="E45" s="6" t="s">
         <v>21</v>
       </c>
       <c r="F45" s="6" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="G45" s="14" t="s">
         <v>13</v>
       </c>
-      <c r="H45" s="18"/>
+      <c r="H45" s="17"/>
     </row>
     <row r="46" spans="1:8" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A46" s="32" t="s">
+      <c r="A46" s="30" t="s">
+        <v>161</v>
+      </c>
+      <c r="B46" s="6" t="s">
+        <v>119</v>
+      </c>
+      <c r="C46" s="6" t="s">
+        <v>159</v>
+      </c>
+      <c r="D46" s="6" t="s">
         <v>162</v>
       </c>
-      <c r="B46" s="6" t="s">
-        <v>120</v>
-      </c>
-      <c r="C46" s="6" t="s">
-        <v>160</v>
-      </c>
-      <c r="D46" s="6" t="s">
+      <c r="E46" s="6" t="s">
         <v>163</v>
       </c>
-      <c r="E46" s="6" t="s">
+      <c r="F46" s="6" t="s">
         <v>164</v>
       </c>
-      <c r="F46" s="6" t="s">
+      <c r="G46" s="14" t="s">
+        <v>13</v>
+      </c>
+      <c r="H46" s="17"/>
+    </row>
+    <row r="47" spans="1:8" ht="34.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A47" s="40" t="s">
         <v>165</v>
       </c>
-      <c r="G46" s="14" t="s">
-        <v>13</v>
-      </c>
-      <c r="H46" s="18"/>
-    </row>
-    <row r="47" spans="1:8" ht="34.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A47" s="42" t="s">
+      <c r="B47" s="40"/>
+      <c r="C47" s="40"/>
+      <c r="D47" s="40"/>
+      <c r="E47" s="40"/>
+      <c r="F47" s="40"/>
+      <c r="G47" s="40"/>
+      <c r="H47" s="16"/>
+    </row>
+    <row r="48" spans="1:8" ht="49.5" x14ac:dyDescent="0.25">
+      <c r="A48" s="30" t="s">
         <v>166</v>
       </c>
-      <c r="B47" s="42"/>
-      <c r="C47" s="42"/>
-      <c r="D47" s="42"/>
-      <c r="E47" s="42"/>
-      <c r="F47" s="42"/>
-      <c r="G47" s="42"/>
-      <c r="H47" s="16"/>
-    </row>
-    <row r="48" spans="1:8" ht="49.5" x14ac:dyDescent="0.25">
-      <c r="A48" s="32" t="s">
+      <c r="B48" s="6" t="s">
         <v>167</v>
       </c>
-      <c r="B48" s="6" t="s">
+      <c r="C48" s="6" t="s">
         <v>168</v>
       </c>
-      <c r="C48" s="6" t="s">
+      <c r="D48" s="6" t="s">
         <v>169</v>
-      </c>
-      <c r="D48" s="6" t="s">
-        <v>170</v>
       </c>
       <c r="E48" s="6" t="s">
         <v>17</v>
       </c>
       <c r="F48" s="6" t="s">
+        <v>170</v>
+      </c>
+      <c r="G48" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="H48" s="15"/>
+    </row>
+    <row r="49" spans="1:8" ht="49.5" x14ac:dyDescent="0.25">
+      <c r="A49" s="30" t="s">
         <v>171</v>
       </c>
-      <c r="G48" s="12" t="s">
-        <v>13</v>
-      </c>
-      <c r="H48" s="15"/>
-    </row>
-    <row r="49" spans="1:8" ht="49.5" x14ac:dyDescent="0.25">
-      <c r="A49" s="32" t="s">
+      <c r="B49" s="6" t="s">
+        <v>167</v>
+      </c>
+      <c r="C49" s="6" t="s">
         <v>172</v>
       </c>
-      <c r="B49" s="6" t="s">
-        <v>168</v>
-      </c>
-      <c r="C49" s="6" t="s">
+      <c r="D49" s="6" t="s">
         <v>173</v>
       </c>
-      <c r="D49" s="6" t="s">
+      <c r="E49" s="6" t="s">
         <v>174</v>
       </c>
-      <c r="E49" s="6" t="s">
+      <c r="F49" s="6" t="s">
         <v>175</v>
       </c>
-      <c r="F49" s="6" t="s">
+      <c r="G49" s="14" t="s">
+        <v>13</v>
+      </c>
+      <c r="H49" s="17"/>
+    </row>
+    <row r="50" spans="1:8" ht="49.5" x14ac:dyDescent="0.25">
+      <c r="A50" s="30" t="s">
         <v>176</v>
       </c>
-      <c r="G49" s="14" t="s">
-        <v>13</v>
-      </c>
-      <c r="H49" s="18"/>
-    </row>
-    <row r="50" spans="1:8" ht="49.5" x14ac:dyDescent="0.25">
-      <c r="A50" s="32" t="s">
+      <c r="B50" s="6" t="s">
+        <v>167</v>
+      </c>
+      <c r="C50" s="6" t="s">
+        <v>172</v>
+      </c>
+      <c r="D50" s="6" t="s">
         <v>177</v>
-      </c>
-      <c r="B50" s="6" t="s">
-        <v>168</v>
-      </c>
-      <c r="C50" s="6" t="s">
-        <v>173</v>
-      </c>
-      <c r="D50" s="6" t="s">
-        <v>178</v>
       </c>
       <c r="E50" s="6" t="s">
         <v>17</v>
       </c>
       <c r="F50" s="6" t="s">
+        <v>178</v>
+      </c>
+      <c r="G50" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="H50" s="15"/>
+    </row>
+    <row r="51" spans="1:8" ht="82.5" x14ac:dyDescent="0.25">
+      <c r="A51" s="30" t="s">
         <v>179</v>
       </c>
-      <c r="G50" s="12" t="s">
-        <v>13</v>
-      </c>
-      <c r="H50" s="15"/>
-    </row>
-    <row r="51" spans="1:8" ht="82.5" x14ac:dyDescent="0.25">
-      <c r="A51" s="32" t="s">
+      <c r="B51" s="6" t="s">
+        <v>167</v>
+      </c>
+      <c r="C51" s="6" t="s">
         <v>180</v>
       </c>
-      <c r="B51" s="6" t="s">
-        <v>168</v>
-      </c>
-      <c r="C51" s="6" t="s">
+      <c r="D51" s="6" t="s">
         <v>181</v>
       </c>
-      <c r="D51" s="6" t="s">
+      <c r="E51" s="6" t="s">
         <v>182</v>
       </c>
-      <c r="E51" s="6" t="s">
+      <c r="F51" s="6" t="s">
         <v>183</v>
       </c>
-      <c r="F51" s="6" t="s">
+      <c r="G51" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="H51" s="15"/>
+    </row>
+    <row r="52" spans="1:8" ht="49.5" x14ac:dyDescent="0.25">
+      <c r="A52" s="30" t="s">
         <v>184</v>
       </c>
-      <c r="G51" s="12" t="s">
-        <v>13</v>
-      </c>
-      <c r="H51" s="15"/>
-    </row>
-    <row r="52" spans="1:8" ht="49.5" x14ac:dyDescent="0.25">
-      <c r="A52" s="32" t="s">
+      <c r="B52" s="6" t="s">
+        <v>167</v>
+      </c>
+      <c r="C52" s="6" t="s">
         <v>185</v>
       </c>
-      <c r="B52" s="6" t="s">
-        <v>168</v>
-      </c>
-      <c r="C52" s="6" t="s">
+      <c r="D52" s="6" t="s">
         <v>186</v>
       </c>
-      <c r="D52" s="6" t="s">
+      <c r="E52" s="6" t="s">
         <v>187</v>
       </c>
-      <c r="E52" s="6" t="s">
+      <c r="F52" s="6" t="s">
         <v>188</v>
       </c>
-      <c r="F52" s="6" t="s">
+      <c r="G52" s="14" t="s">
+        <v>13</v>
+      </c>
+      <c r="H52" s="17"/>
+    </row>
+    <row r="53" spans="1:8" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A53" s="42" t="s">
         <v>189</v>
       </c>
-      <c r="G52" s="14" t="s">
-        <v>13</v>
-      </c>
-      <c r="H52" s="18"/>
-    </row>
-    <row r="53" spans="1:8" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A53" s="43" t="s">
+      <c r="B53" s="42"/>
+      <c r="C53" s="42"/>
+      <c r="D53" s="42"/>
+      <c r="E53" s="42"/>
+      <c r="F53" s="42"/>
+      <c r="G53" s="43"/>
+      <c r="H53" s="13"/>
+    </row>
+    <row r="54" spans="1:8" ht="66" x14ac:dyDescent="0.25">
+      <c r="A54" s="30" t="s">
         <v>190</v>
       </c>
-      <c r="B53" s="43"/>
-      <c r="C53" s="43"/>
-      <c r="D53" s="43"/>
-      <c r="E53" s="43"/>
-      <c r="F53" s="43"/>
-      <c r="G53" s="44"/>
-      <c r="H53" s="17"/>
-    </row>
-    <row r="54" spans="1:8" ht="66" x14ac:dyDescent="0.25">
-      <c r="A54" s="32" t="s">
+      <c r="B54" s="7" t="s">
         <v>191</v>
       </c>
-      <c r="B54" s="7" t="s">
+      <c r="C54" s="7" t="s">
         <v>192</v>
       </c>
-      <c r="C54" s="7" t="s">
+      <c r="D54" s="7" t="s">
         <v>193</v>
       </c>
-      <c r="D54" s="7" t="s">
+      <c r="E54" s="7" t="s">
         <v>194</v>
       </c>
-      <c r="E54" s="7" t="s">
+      <c r="F54" s="7" t="s">
         <v>195</v>
       </c>
-      <c r="F54" s="7" t="s">
+      <c r="G54" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="H54" s="15"/>
+    </row>
+    <row r="55" spans="1:8" ht="33" x14ac:dyDescent="0.25">
+      <c r="A55" s="30" t="s">
         <v>196</v>
       </c>
-      <c r="G54" s="12" t="s">
-        <v>13</v>
-      </c>
-      <c r="H54" s="15"/>
-    </row>
-    <row r="55" spans="1:8" ht="33" x14ac:dyDescent="0.25">
-      <c r="A55" s="32" t="s">
+      <c r="B55" s="7" t="s">
+        <v>191</v>
+      </c>
+      <c r="C55" s="7" t="s">
+        <v>192</v>
+      </c>
+      <c r="D55" s="7" t="s">
         <v>197</v>
       </c>
-      <c r="B55" s="7" t="s">
+      <c r="E55" s="7" t="s">
+        <v>198</v>
+      </c>
+      <c r="F55" s="7" t="s">
+        <v>199</v>
+      </c>
+      <c r="G55" s="14" t="s">
+        <v>13</v>
+      </c>
+      <c r="H55" s="17"/>
+    </row>
+    <row r="56" spans="1:8" ht="33" x14ac:dyDescent="0.25">
+      <c r="A56" s="30" t="s">
+        <v>200</v>
+      </c>
+      <c r="B56" s="7" t="s">
+        <v>191</v>
+      </c>
+      <c r="C56" s="7" t="s">
         <v>192</v>
       </c>
-      <c r="C55" s="7" t="s">
-        <v>193</v>
-      </c>
-      <c r="D55" s="7" t="s">
-        <v>198</v>
-      </c>
-      <c r="E55" s="7" t="s">
-        <v>199</v>
-      </c>
-      <c r="F55" s="7" t="s">
-        <v>200</v>
-      </c>
-      <c r="G55" s="14" t="s">
-        <v>13</v>
-      </c>
-      <c r="H55" s="18"/>
-    </row>
-    <row r="56" spans="1:8" ht="33" x14ac:dyDescent="0.25">
-      <c r="A56" s="32" t="s">
+      <c r="D56" s="7" t="s">
         <v>201</v>
       </c>
-      <c r="B56" s="7" t="s">
-        <v>192</v>
-      </c>
-      <c r="C56" s="7" t="s">
-        <v>193</v>
-      </c>
-      <c r="D56" s="7" t="s">
+      <c r="E56" s="7" t="s">
         <v>202</v>
       </c>
-      <c r="E56" s="7" t="s">
+      <c r="F56" s="7" t="s">
         <v>203</v>
       </c>
-      <c r="F56" s="7" t="s">
+      <c r="G56" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="H56" s="15"/>
+    </row>
+    <row r="57" spans="1:8" ht="40.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A57" s="42" t="s">
         <v>204</v>
       </c>
-      <c r="G56" s="12" t="s">
-        <v>13</v>
-      </c>
-      <c r="H56" s="15"/>
-    </row>
-    <row r="57" spans="1:8" ht="40.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A57" s="43" t="s">
+      <c r="B57" s="42"/>
+      <c r="C57" s="42"/>
+      <c r="D57" s="42"/>
+      <c r="E57" s="42"/>
+      <c r="F57" s="42"/>
+      <c r="G57" s="43"/>
+      <c r="H57" s="25"/>
+    </row>
+    <row r="58" spans="1:8" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A58" s="30" t="s">
         <v>205</v>
       </c>
-      <c r="B57" s="43"/>
-      <c r="C57" s="43"/>
-      <c r="D57" s="43"/>
-      <c r="E57" s="43"/>
-      <c r="F57" s="43"/>
-      <c r="G57" s="44"/>
-      <c r="H57" s="26"/>
-    </row>
-    <row r="58" spans="1:8" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A58" s="32" t="s">
+      <c r="B58" s="6" t="s">
         <v>206</v>
       </c>
-      <c r="B58" s="6" t="s">
+      <c r="C58" s="6" t="s">
         <v>207</v>
       </c>
-      <c r="C58" s="6" t="s">
+      <c r="D58" s="6" t="s">
         <v>208</v>
-      </c>
-      <c r="D58" s="6" t="s">
-        <v>209</v>
       </c>
       <c r="E58" s="6" t="s">
         <v>17</v>
       </c>
       <c r="F58" s="6" t="s">
+        <v>209</v>
+      </c>
+      <c r="G58" s="28" t="s">
+        <v>13</v>
+      </c>
+      <c r="H58" s="17"/>
+    </row>
+    <row r="59" spans="1:8" ht="49.5" x14ac:dyDescent="0.25">
+      <c r="A59" s="30" t="s">
         <v>210</v>
       </c>
-      <c r="G58" s="30" t="s">
-        <v>13</v>
-      </c>
-      <c r="H58" s="18"/>
-    </row>
-    <row r="59" spans="1:8" ht="49.5" x14ac:dyDescent="0.25">
-      <c r="A59" s="32" t="s">
+      <c r="B59" s="6" t="s">
+        <v>206</v>
+      </c>
+      <c r="C59" s="6" t="s">
         <v>211</v>
       </c>
-      <c r="B59" s="6" t="s">
-        <v>207</v>
-      </c>
-      <c r="C59" s="6" t="s">
+      <c r="D59" s="6" t="s">
         <v>212</v>
-      </c>
-      <c r="D59" s="6" t="s">
-        <v>213</v>
       </c>
       <c r="E59" s="6" t="s">
         <v>17</v>
       </c>
       <c r="F59" s="6" t="s">
+        <v>213</v>
+      </c>
+      <c r="G59" s="28" t="s">
+        <v>13</v>
+      </c>
+      <c r="H59" s="17"/>
+    </row>
+    <row r="60" spans="1:8" ht="66" x14ac:dyDescent="0.25">
+      <c r="A60" s="30" t="s">
         <v>214</v>
       </c>
-      <c r="G59" s="30" t="s">
-        <v>13</v>
-      </c>
-      <c r="H59" s="18"/>
-    </row>
-    <row r="60" spans="1:8" ht="66" x14ac:dyDescent="0.25">
-      <c r="A60" s="32" t="s">
+      <c r="B60" s="6" t="s">
+        <v>206</v>
+      </c>
+      <c r="C60" s="6" t="s">
         <v>215</v>
       </c>
-      <c r="B60" s="6" t="s">
-        <v>207</v>
-      </c>
-      <c r="C60" s="6" t="s">
+      <c r="D60" s="6" t="s">
         <v>216</v>
-      </c>
-      <c r="D60" s="6" t="s">
-        <v>217</v>
       </c>
       <c r="E60" s="6" t="s">
         <v>17</v>
       </c>
       <c r="F60" s="6" t="s">
+        <v>217</v>
+      </c>
+      <c r="G60" s="28" t="s">
+        <v>13</v>
+      </c>
+      <c r="H60" s="17"/>
+    </row>
+    <row r="61" spans="1:8" ht="49.5" x14ac:dyDescent="0.25">
+      <c r="A61" s="30" t="s">
         <v>218</v>
       </c>
-      <c r="G60" s="30" t="s">
-        <v>13</v>
-      </c>
-      <c r="H60" s="18"/>
-    </row>
-    <row r="61" spans="1:8" ht="49.5" x14ac:dyDescent="0.25">
-      <c r="A61" s="32" t="s">
+      <c r="B61" s="6" t="s">
+        <v>206</v>
+      </c>
+      <c r="C61" s="6" t="s">
         <v>219</v>
       </c>
-      <c r="B61" s="6" t="s">
-        <v>207</v>
-      </c>
-      <c r="C61" s="6" t="s">
+      <c r="D61" s="6" t="s">
         <v>220</v>
-      </c>
-      <c r="D61" s="6" t="s">
-        <v>221</v>
       </c>
       <c r="E61" s="6" t="s">
         <v>17</v>
       </c>
       <c r="F61" s="6" t="s">
+        <v>221</v>
+      </c>
+      <c r="G61" s="28" t="s">
+        <v>13</v>
+      </c>
+      <c r="H61" s="17"/>
+    </row>
+    <row r="62" spans="1:8" ht="49.5" x14ac:dyDescent="0.25">
+      <c r="A62" s="30" t="s">
         <v>222</v>
       </c>
-      <c r="G61" s="30" t="s">
-        <v>13</v>
-      </c>
-      <c r="H61" s="18"/>
-    </row>
-    <row r="62" spans="1:8" ht="49.5" x14ac:dyDescent="0.25">
-      <c r="A62" s="32" t="s">
+      <c r="B62" s="6" t="s">
+        <v>206</v>
+      </c>
+      <c r="C62" s="6" t="s">
         <v>223</v>
       </c>
-      <c r="B62" s="6" t="s">
-        <v>207</v>
-      </c>
-      <c r="C62" s="6" t="s">
+      <c r="D62" s="6" t="s">
         <v>224</v>
       </c>
-      <c r="D62" s="6" t="s">
+      <c r="E62" s="6" t="s">
         <v>225</v>
       </c>
-      <c r="E62" s="6" t="s">
+      <c r="F62" s="6" t="s">
         <v>226</v>
       </c>
-      <c r="F62" s="6" t="s">
+      <c r="G62" s="28" t="s">
+        <v>13</v>
+      </c>
+      <c r="H62" s="17"/>
+    </row>
+    <row r="63" spans="1:8" ht="33" x14ac:dyDescent="0.25">
+      <c r="A63" s="30" t="s">
         <v>227</v>
       </c>
-      <c r="G62" s="30" t="s">
-        <v>13</v>
-      </c>
-      <c r="H62" s="18"/>
-    </row>
-    <row r="63" spans="1:8" ht="33" x14ac:dyDescent="0.25">
-      <c r="A63" s="32" t="s">
+      <c r="B63" s="6" t="s">
+        <v>206</v>
+      </c>
+      <c r="C63" s="6" t="s">
+        <v>223</v>
+      </c>
+      <c r="D63" s="6" t="s">
         <v>228</v>
       </c>
-      <c r="B63" s="6" t="s">
-        <v>207</v>
-      </c>
-      <c r="C63" s="6" t="s">
-        <v>224</v>
-      </c>
-      <c r="D63" s="6" t="s">
+      <c r="E63" s="6" t="s">
         <v>229</v>
       </c>
-      <c r="E63" s="6" t="s">
+      <c r="F63" s="6" t="s">
         <v>230</v>
       </c>
-      <c r="F63" s="6" t="s">
+      <c r="G63" s="28" t="s">
+        <v>13</v>
+      </c>
+      <c r="H63" s="17"/>
+    </row>
+    <row r="64" spans="1:8" ht="49.5" x14ac:dyDescent="0.25">
+      <c r="A64" s="30" t="s">
         <v>231</v>
       </c>
-      <c r="G63" s="30" t="s">
-        <v>13</v>
-      </c>
-      <c r="H63" s="18"/>
-    </row>
-    <row r="64" spans="1:8" ht="49.5" x14ac:dyDescent="0.25">
-      <c r="A64" s="32" t="s">
+      <c r="B64" s="6" t="s">
+        <v>206</v>
+      </c>
+      <c r="C64" s="6" t="s">
         <v>232</v>
       </c>
-      <c r="B64" s="6" t="s">
-        <v>207</v>
-      </c>
-      <c r="C64" s="6" t="s">
+      <c r="D64" s="6" t="s">
         <v>233</v>
-      </c>
-      <c r="D64" s="6" t="s">
-        <v>234</v>
       </c>
       <c r="E64" s="6" t="s">
         <v>17</v>
       </c>
       <c r="F64" s="6" t="s">
+        <v>234</v>
+      </c>
+      <c r="G64" s="28" t="s">
+        <v>13</v>
+      </c>
+      <c r="H64" s="13"/>
+    </row>
+    <row r="65" spans="1:8" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A65" s="44" t="s">
         <v>235</v>
       </c>
-      <c r="G64" s="30" t="s">
-        <v>13</v>
-      </c>
-      <c r="H64" s="13"/>
-    </row>
-    <row r="65" spans="1:8" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A65" s="45" t="s">
+      <c r="B65" s="44"/>
+      <c r="C65" s="44"/>
+      <c r="D65" s="44"/>
+      <c r="E65" s="44"/>
+      <c r="F65" s="44"/>
+      <c r="G65" s="44"/>
+      <c r="H65" s="13"/>
+    </row>
+    <row r="66" spans="1:8" ht="33" x14ac:dyDescent="0.25">
+      <c r="A66" s="30" t="s">
         <v>236</v>
       </c>
-      <c r="B65" s="45"/>
-      <c r="C65" s="45"/>
-      <c r="D65" s="45"/>
-      <c r="E65" s="45"/>
-      <c r="F65" s="45"/>
-      <c r="G65" s="45"/>
-      <c r="H65" s="17"/>
-    </row>
-    <row r="66" spans="1:8" ht="33" x14ac:dyDescent="0.25">
-      <c r="A66" s="32" t="s">
+      <c r="B66" s="6" t="s">
         <v>237</v>
       </c>
-      <c r="B66" s="6" t="s">
+      <c r="C66" s="6" t="s">
         <v>238</v>
       </c>
-      <c r="C66" s="6" t="s">
+      <c r="D66" s="6" t="s">
         <v>239</v>
       </c>
-      <c r="D66" s="6" t="s">
+      <c r="E66" s="6" t="s">
         <v>240</v>
       </c>
-      <c r="E66" s="6" t="s">
+      <c r="F66" s="6" t="s">
         <v>241</v>
       </c>
-      <c r="F66" s="6" t="s">
+      <c r="G66" s="28" t="s">
+        <v>13</v>
+      </c>
+      <c r="H66" s="17"/>
+    </row>
+    <row r="67" spans="1:8" ht="49.5" x14ac:dyDescent="0.25">
+      <c r="A67" s="30" t="s">
         <v>242</v>
       </c>
-      <c r="G66" s="30" t="s">
-        <v>13</v>
-      </c>
-      <c r="H66" s="18"/>
-    </row>
-    <row r="67" spans="1:8" ht="49.5" x14ac:dyDescent="0.25">
-      <c r="A67" s="32" t="s">
+      <c r="B67" s="6" t="s">
+        <v>237</v>
+      </c>
+      <c r="C67" s="6" t="s">
         <v>243</v>
       </c>
-      <c r="B67" s="6" t="s">
-        <v>238</v>
-      </c>
-      <c r="C67" s="6" t="s">
+      <c r="D67" s="6" t="s">
         <v>244</v>
       </c>
-      <c r="D67" s="6" t="s">
+      <c r="E67" s="6" t="s">
         <v>245</v>
       </c>
-      <c r="E67" s="6" t="s">
+      <c r="F67" s="6" t="s">
         <v>246</v>
       </c>
-      <c r="F67" s="6" t="s">
+      <c r="G67" s="28" t="s">
+        <v>13</v>
+      </c>
+      <c r="H67" s="17"/>
+    </row>
+    <row r="68" spans="1:8" ht="33" x14ac:dyDescent="0.25">
+      <c r="A68" s="30" t="s">
         <v>247</v>
       </c>
-      <c r="G67" s="30" t="s">
-        <v>13</v>
-      </c>
-      <c r="H67" s="18"/>
-    </row>
-    <row r="68" spans="1:8" ht="33" x14ac:dyDescent="0.25">
-      <c r="A68" s="32" t="s">
+      <c r="B68" s="6" t="s">
+        <v>237</v>
+      </c>
+      <c r="C68" s="6" t="s">
+        <v>243</v>
+      </c>
+      <c r="D68" s="6" t="s">
         <v>248</v>
       </c>
-      <c r="B68" s="6" t="s">
-        <v>238</v>
-      </c>
-      <c r="C68" s="6" t="s">
-        <v>244</v>
-      </c>
-      <c r="D68" s="6" t="s">
+      <c r="E68" s="6" t="s">
         <v>249</v>
       </c>
-      <c r="E68" s="6" t="s">
+      <c r="F68" s="6" t="s">
         <v>250</v>
       </c>
-      <c r="F68" s="6" t="s">
+      <c r="G68" s="28" t="s">
+        <v>13</v>
+      </c>
+      <c r="H68" s="17"/>
+    </row>
+    <row r="69" spans="1:8" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A69" s="44" t="s">
         <v>251</v>
       </c>
-      <c r="G68" s="30" t="s">
-        <v>13</v>
-      </c>
-      <c r="H68" s="18"/>
-    </row>
-    <row r="69" spans="1:8" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A69" s="45" t="s">
+      <c r="B69" s="44"/>
+      <c r="C69" s="44"/>
+      <c r="D69" s="44"/>
+      <c r="E69" s="44"/>
+      <c r="F69" s="44"/>
+      <c r="G69" s="44"/>
+      <c r="H69" s="13"/>
+    </row>
+    <row r="70" spans="1:8" ht="66" x14ac:dyDescent="0.25">
+      <c r="A70" s="30" t="s">
         <v>252</v>
       </c>
-      <c r="B69" s="45"/>
-      <c r="C69" s="45"/>
-      <c r="D69" s="45"/>
-      <c r="E69" s="45"/>
-      <c r="F69" s="45"/>
-      <c r="G69" s="45"/>
-      <c r="H69" s="17"/>
-    </row>
-    <row r="70" spans="1:8" ht="66" x14ac:dyDescent="0.25">
-      <c r="A70" s="32" t="s">
+      <c r="B70" s="6" t="s">
         <v>253</v>
-      </c>
-      <c r="B70" s="6" t="s">
-        <v>254</v>
       </c>
       <c r="C70" s="6" t="s">
         <v>9</v>
       </c>
       <c r="D70" s="6" t="s">
+        <v>254</v>
+      </c>
+      <c r="E70" s="6" t="s">
         <v>255</v>
       </c>
-      <c r="E70" s="6" t="s">
+      <c r="F70" s="6" t="s">
         <v>256</v>
       </c>
-      <c r="F70" s="6" t="s">
+      <c r="G70" s="28" t="s">
+        <v>13</v>
+      </c>
+      <c r="H70" s="17"/>
+    </row>
+    <row r="71" spans="1:8" ht="49.5" x14ac:dyDescent="0.25">
+      <c r="A71" s="30" t="s">
         <v>257</v>
       </c>
-      <c r="G70" s="30" t="s">
-        <v>13</v>
-      </c>
-      <c r="H70" s="18"/>
-    </row>
-    <row r="71" spans="1:8" ht="49.5" x14ac:dyDescent="0.25">
-      <c r="A71" s="32" t="s">
+      <c r="B71" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="C71" s="6" t="s">
         <v>258</v>
       </c>
-      <c r="B71" s="6" t="s">
-        <v>254</v>
-      </c>
-      <c r="C71" s="6" t="s">
+      <c r="D71" s="6" t="s">
         <v>259</v>
       </c>
-      <c r="D71" s="6" t="s">
+      <c r="E71" s="6" t="s">
         <v>260</v>
       </c>
-      <c r="E71" s="6" t="s">
+      <c r="F71" s="6" t="s">
         <v>261</v>
       </c>
-      <c r="F71" s="6" t="s">
+      <c r="G71" s="28" t="s">
+        <v>13</v>
+      </c>
+      <c r="H71" s="17"/>
+    </row>
+    <row r="72" spans="1:8" ht="33" x14ac:dyDescent="0.25">
+      <c r="A72" s="30" t="s">
         <v>262</v>
       </c>
-      <c r="G71" s="30" t="s">
-        <v>13</v>
-      </c>
-      <c r="H71" s="18"/>
-    </row>
-    <row r="72" spans="1:8" ht="33" x14ac:dyDescent="0.25">
-      <c r="A72" s="32" t="s">
+      <c r="B72" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="C72" s="6" t="s">
+        <v>258</v>
+      </c>
+      <c r="D72" s="6" t="s">
         <v>263</v>
       </c>
-      <c r="B72" s="6" t="s">
-        <v>254</v>
-      </c>
-      <c r="C72" s="6" t="s">
-        <v>259</v>
-      </c>
-      <c r="D72" s="6" t="s">
+      <c r="E72" s="6" t="s">
         <v>264</v>
       </c>
-      <c r="E72" s="6" t="s">
+      <c r="F72" s="6" t="s">
         <v>265</v>
       </c>
-      <c r="F72" s="6" t="s">
+      <c r="G72" s="28" t="s">
+        <v>13</v>
+      </c>
+      <c r="H72" s="17"/>
+    </row>
+    <row r="73" spans="1:8" ht="66" x14ac:dyDescent="0.25">
+      <c r="A73" s="30" t="s">
         <v>266</v>
       </c>
-      <c r="G72" s="30" t="s">
-        <v>13</v>
-      </c>
-      <c r="H72" s="18"/>
-    </row>
-    <row r="73" spans="1:8" ht="66" x14ac:dyDescent="0.25">
-      <c r="A73" s="32" t="s">
+      <c r="B73" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="C73" s="6" t="s">
         <v>267</v>
       </c>
-      <c r="B73" s="6" t="s">
-        <v>254</v>
-      </c>
-      <c r="C73" s="6" t="s">
+      <c r="D73" s="6" t="s">
         <v>268</v>
-      </c>
-      <c r="D73" s="6" t="s">
-        <v>269</v>
       </c>
       <c r="E73" s="6" t="s">
         <v>17</v>
       </c>
       <c r="F73" s="6" t="s">
-        <v>270</v>
-      </c>
-      <c r="G73" s="30" t="s">
+        <v>269</v>
+      </c>
+      <c r="G73" s="28" t="s">
         <v>13</v>
       </c>
       <c r="H73" s="13"/>
     </row>
     <row r="74" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A74" s="37"/>
+      <c r="A74" s="35"/>
     </row>
     <row r="75" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A75" s="8"/>
@@ -5091,14 +5108,170 @@
     <mergeCell ref="A57:G57"/>
     <mergeCell ref="A65:G65"/>
     <mergeCell ref="A69:G69"/>
+    <mergeCell ref="A4:G4"/>
+    <mergeCell ref="A34:G34"/>
     <mergeCell ref="A1:G2"/>
-    <mergeCell ref="A3:G3"/>
     <mergeCell ref="A9:G9"/>
     <mergeCell ref="A16:G16"/>
     <mergeCell ref="A24:G24"/>
-    <mergeCell ref="A34:G34"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D9F88A26-56FA-4B1C-97DA-FDAD85DDFD4F}">
+  <dimension ref="A1:G11"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:7" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="A1" s="46" t="s">
+        <v>272</v>
+      </c>
+      <c r="B1" s="46"/>
+      <c r="C1" s="46"/>
+      <c r="D1" s="46"/>
+      <c r="E1" s="46"/>
+      <c r="F1" s="46"/>
+      <c r="G1" s="46"/>
+    </row>
+    <row r="2" spans="1:7" ht="24" x14ac:dyDescent="0.25">
+      <c r="A2" s="45" t="s">
+        <v>26</v>
+      </c>
+      <c r="B2" s="45"/>
+      <c r="C2" s="45"/>
+      <c r="D2" s="45"/>
+      <c r="E2" s="45"/>
+      <c r="F2" s="45"/>
+      <c r="G2" s="45"/>
+    </row>
+    <row r="3" spans="1:7" ht="24" x14ac:dyDescent="0.25">
+      <c r="A3" s="45" t="s">
+        <v>273</v>
+      </c>
+      <c r="B3" s="45"/>
+      <c r="C3" s="45"/>
+      <c r="D3" s="45"/>
+      <c r="E3" s="45"/>
+      <c r="F3" s="45"/>
+      <c r="G3" s="45"/>
+    </row>
+    <row r="4" spans="1:7" ht="24" x14ac:dyDescent="0.25">
+      <c r="A4" s="45" t="s">
+        <v>274</v>
+      </c>
+      <c r="B4" s="45"/>
+      <c r="C4" s="45"/>
+      <c r="D4" s="45"/>
+      <c r="E4" s="45"/>
+      <c r="F4" s="45"/>
+      <c r="G4" s="45"/>
+    </row>
+    <row r="5" spans="1:7" ht="24" x14ac:dyDescent="0.25">
+      <c r="A5" s="45" t="s">
+        <v>275</v>
+      </c>
+      <c r="B5" s="45"/>
+      <c r="C5" s="45"/>
+      <c r="D5" s="45"/>
+      <c r="E5" s="45"/>
+      <c r="F5" s="45"/>
+      <c r="G5" s="45"/>
+    </row>
+    <row r="6" spans="1:7" ht="24" x14ac:dyDescent="0.25">
+      <c r="A6" s="45" t="s">
+        <v>276</v>
+      </c>
+      <c r="B6" s="45"/>
+      <c r="C6" s="45"/>
+      <c r="D6" s="45"/>
+      <c r="E6" s="45"/>
+      <c r="F6" s="45"/>
+      <c r="G6" s="45"/>
+    </row>
+    <row r="7" spans="1:7" ht="24" x14ac:dyDescent="0.25">
+      <c r="A7" s="45" t="s">
+        <v>277</v>
+      </c>
+      <c r="B7" s="45"/>
+      <c r="C7" s="45"/>
+      <c r="D7" s="45"/>
+      <c r="E7" s="45"/>
+      <c r="F7" s="45"/>
+      <c r="G7" s="45"/>
+    </row>
+    <row r="8" spans="1:7" ht="24" x14ac:dyDescent="0.25">
+      <c r="A8" s="45" t="s">
+        <v>278</v>
+      </c>
+      <c r="B8" s="45"/>
+      <c r="C8" s="45"/>
+      <c r="D8" s="45"/>
+      <c r="E8" s="45"/>
+      <c r="F8" s="45"/>
+      <c r="G8" s="45"/>
+    </row>
+    <row r="9" spans="1:7" ht="24" x14ac:dyDescent="0.25">
+      <c r="A9" s="45" t="s">
+        <v>279</v>
+      </c>
+      <c r="B9" s="45"/>
+      <c r="C9" s="45"/>
+      <c r="D9" s="45"/>
+      <c r="E9" s="45"/>
+      <c r="F9" s="45"/>
+      <c r="G9" s="45"/>
+    </row>
+    <row r="10" spans="1:7" ht="24" x14ac:dyDescent="0.25">
+      <c r="A10" s="45" t="s">
+        <v>280</v>
+      </c>
+      <c r="B10" s="45"/>
+      <c r="C10" s="45"/>
+      <c r="D10" s="45"/>
+      <c r="E10" s="45"/>
+      <c r="F10" s="45"/>
+      <c r="G10" s="45"/>
+    </row>
+    <row r="11" spans="1:7" ht="24" x14ac:dyDescent="0.25">
+      <c r="A11" s="45" t="s">
+        <v>281</v>
+      </c>
+      <c r="B11" s="45"/>
+      <c r="C11" s="45"/>
+      <c r="D11" s="45"/>
+      <c r="E11" s="45"/>
+      <c r="F11" s="45"/>
+      <c r="G11" s="45"/>
+    </row>
+  </sheetData>
+  <mergeCells count="11">
+    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A2:G2"/>
+    <mergeCell ref="A4:G4"/>
+    <mergeCell ref="A5:G5"/>
+    <mergeCell ref="A6:G6"/>
+    <mergeCell ref="A3:G3"/>
+    <mergeCell ref="A7:G7"/>
+    <mergeCell ref="A8:G8"/>
+    <mergeCell ref="A9:G9"/>
+    <mergeCell ref="A10:G10"/>
+    <mergeCell ref="A11:G11"/>
+  </mergeCells>
+  <hyperlinks>
+    <hyperlink ref="A3:G3" location="_2._Main_Menu_Module" display="_2._Main_Menu_Module" xr:uid="{D03A7ECE-9DBC-4B77-A71C-4139FC2DB29D}"/>
+    <hyperlink ref="A2:G2" location="Sheet1!A1" display="Sheet1!A1" xr:uid="{BBC754C8-FC77-46C2-9659-9B39956108A7}"/>
+    <hyperlink ref="A4:G4" location="_3._Story_Module" display="_3._Story_Module" xr:uid="{AD9B4D55-86F9-49DE-9642-607455049298}"/>
+    <hyperlink ref="A5:G5" location="_4._Size_Selection_Module" display="_4._Size_Selection_Module" xr:uid="{56075561-937F-4DEC-B4F6-F7194D432EC6}"/>
+    <hyperlink ref="A6:G6" location="_5._Game_Core_Module" display="_5._Game_Core_Module" xr:uid="{B4EA0AC3-0FDA-46B3-AF3E-F0EAD4A1208F}"/>
+    <hyperlink ref="A7:G7" location="_6._Maze_Generation_Module" display="_6._Maze_Generation_Module" xr:uid="{C0F81DF7-9C2F-4C75-86DF-7339DFEB9CF2}"/>
+    <hyperlink ref="A8:G8" location="_7._Player_Module" display="_7._Player_Module" xr:uid="{C1A59AB6-5B86-4616-A51D-47F2977F85DD}"/>
+    <hyperlink ref="A9:G9" location="_8._Timer_System_Module" display="_8._Timer_System_Module" xr:uid="{3B24A5E7-CA16-4B08-A0B0-044A0396F9EE}"/>
+    <hyperlink ref="A10:G10" location="_9._File_Persistence_Module" display="_9._File_Persistence_Module" xr:uid="{14B59E18-149B-4443-83DE-6043269E7CF1}"/>
+    <hyperlink ref="A11:G11" location="_10._UI_Components_Module" display="_10._UI_Components_Module" xr:uid="{24B204E8-926F-4D8B-8BB2-450526EF7D64}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>